<commit_message>
Point site at pillaiandsons.in
</commit_message>
<xml_diff>
--- a/config/site-config.xlsx
+++ b/config/site-config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\madha\Downloads\pillai-and-sons-motor-company-static-site_3\pillai-and-sons-motor-company\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5DA2732-1698-4B75-8986-F800E7E53787}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5DF9087-1A30-46F8-AE9E-11B7072BA579}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1068,7 +1068,7 @@
     <t>The first row is the site default. These palettes appear in the colour switcher visitors can open from the floating paint icon. The two 'Ink' columns are the darker shades used wherever small text meets the colour — they are what keep the site readable.</t>
   </si>
   <si>
-    <t>https://digitalpillai.github.io/pillai-and-sons</t>
+    <t>https://pillaiandsons.in</t>
   </si>
 </sst>
 </file>

</xml_diff>